<commit_message>
Update error trial indices and adjust trial durations in experiment logic
</commit_message>
<xml_diff>
--- a/error_simpleAI.xlsx
+++ b/error_simpleAI.xlsx
@@ -143,6 +143,9 @@
     <t>Safe</t>
   </si>
   <si>
+    <t>Danger</t>
+  </si>
+  <si>
     <t>Simple_Error2</t>
   </si>
   <si>
@@ -150,9 +153,6 @@
   </si>
   <si>
     <t>Simple_Error4</t>
-  </si>
-  <si>
-    <t>Danger</t>
   </si>
   <si>
     <t>Simple_Error5</t>
@@ -266,7 +266,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Stephanie Merritt" id="{E4E539F2-BE31-9C58-1841-B1F20A33DEB0}"/>
+  <person displayName="Stephanie Merritt" id="{55266F82-3ACA-1C1D-070A-11B6DC084104}"/>
 </personList>
 </file>
 
@@ -750,20 +750,20 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A1" personId="{E4E539F2-BE31-9C58-1841-B1F20A33DEB0}" id="{675377BE-BD21-4BFE-9EB3-33184C02554F}" done="0">
+  <threadedComment ref="A1" personId="{55266F82-3ACA-1C1D-070A-11B6DC084104}" id="{675377BE-BD21-4BFE-9EB3-33184C02554F}" done="0">
     <text xml:space="preserve">Slide names correspond to the images stored in the repository.
 </text>
   </threadedComment>
-  <threadedComment ref="B1" personId="{E4E539F2-BE31-9C58-1841-B1F20A33DEB0}" id="{175DE6AE-A4A4-F0DC-1C56-6A0D66D3CF2D}" done="0">
+  <threadedComment ref="B1" personId="{55266F82-3ACA-1C1D-070A-11B6DC084104}" id="{175DE6AE-A4A4-F0DC-1C56-6A0D66D3CF2D}" done="0">
     <text xml:space="preserve">Number of item in the suitcase
 </text>
   </threadedComment>
-  <threadedComment ref="C1" personId="{E4E539F2-BE31-9C58-1841-B1F20A33DEB0}" id="{46E831AE-9613-FED5-458C-E8A9D3212966}" done="0">
+  <threadedComment ref="C1" personId="{55266F82-3ACA-1C1D-070A-11B6DC084104}" id="{46E831AE-9613-FED5-458C-E8A9D3212966}" done="0">
     <text xml:space="preserve">For images containing weapons, the correct answer was "search."
 For images without weapons, the correct answer was "clear."
 </text>
   </threadedComment>
-  <threadedComment ref="D1" personId="{E4E539F2-BE31-9C58-1841-B1F20A33DEB0}" id="{13027208-6B41-4C90-8CBD-5507B2B2EC29}" done="0">
+  <threadedComment ref="D1" personId="{55266F82-3ACA-1C1D-070A-11B6DC084104}" id="{13027208-6B41-4C90-8CBD-5507B2B2EC29}" done="0">
     <text xml:space="preserve">Classical test theory index of difficulty (the inverse of the percent who answered correctly).
 </text>
   </threadedComment>
@@ -773,8 +773,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col bestFit="1" min="1" max="1" width="14.140625"/>
+  </cols>
   <sheetData>
-    <row r="1" ht="14.25">
+    <row r="1" ht="57">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -814,7 +817,7 @@
         <v>51</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G2" s="7">
         <v>31</v>
@@ -822,7 +825,7 @@
     </row>
     <row r="3" ht="14.25">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" s="4">
         <v>4</v>
@@ -845,7 +848,7 @@
     </row>
     <row r="4" ht="14.25">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" s="4">
         <v>6</v>
@@ -860,7 +863,7 @@
         <v>141</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G4" s="7">
         <v>35</v>
@@ -868,13 +871,13 @@
     </row>
     <row r="5" ht="14.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B5" s="8">
         <v>6</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D5" s="5">
         <v>0.16</v>
@@ -883,7 +886,7 @@
         <v>47</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G5" s="7">
         <v>87</v>
@@ -897,7 +900,7 @@
         <v>6</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D6" s="5">
         <v>0.14000000000000001</v>
@@ -906,7 +909,7 @@
         <v>44</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G6" s="7">
         <v>90</v>
@@ -929,7 +932,7 @@
         <v>46</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G7" s="7">
         <v>103</v>
@@ -943,7 +946,7 @@
         <v>8</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D8" s="5">
         <v>0.20000000000000001</v>
@@ -952,7 +955,7 @@
         <v>56</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G8" s="7">
         <v>84</v>

</xml_diff>